<commit_message>
Fix EN/MN numeric mismatch and XLSX wide format
- Rebuild CSVs from single source with consistent order index
  to ensure EN and MN rows have identical numeric values
- Regenerate XLSX in wide format (years as columns)
- All 52 validation checks now pass

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/school-enrollment-by-level.xlsx
+++ b/data.mn/public/datasets/school-enrollment-by-level.xlsx
@@ -414,306 +414,282 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+          <t>Education Level</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E1" t="n">
+        <v>2013</v>
+      </c>
+      <c r="F1" t="n">
+        <v>2014</v>
+      </c>
+      <c r="G1" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H1" t="n">
+        <v>2016</v>
+      </c>
+      <c r="I1" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J1" t="n">
+        <v>2018</v>
+      </c>
+      <c r="K1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="L1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="M1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="N1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="O1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="P1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Early childhood education</t>
         </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>General education</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Higher education</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Vocational education</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>2010</v>
       </c>
       <c r="B2" t="n">
         <v>157200</v>
       </c>
       <c r="C2" t="n">
+        <v>164300</v>
+      </c>
+      <c r="D2" t="n">
+        <v>181000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>193700</v>
+      </c>
+      <c r="F2" t="n">
+        <v>206600</v>
+      </c>
+      <c r="G2" t="n">
+        <v>225400</v>
+      </c>
+      <c r="H2" t="n">
+        <v>243400</v>
+      </c>
+      <c r="I2" t="n">
+        <v>256700</v>
+      </c>
+      <c r="J2" t="n">
+        <v>261300</v>
+      </c>
+      <c r="K2" t="n">
+        <v>263300</v>
+      </c>
+      <c r="L2" t="n">
+        <v>247000</v>
+      </c>
+      <c r="M2" t="n">
+        <v>191000</v>
+      </c>
+      <c r="N2" t="n">
+        <v>266000</v>
+      </c>
+      <c r="O2" t="n">
+        <v>274200</v>
+      </c>
+      <c r="P2" t="n">
+        <v>264800</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>258800</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>General education</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>512200</v>
-      </c>
-      <c r="D2" t="n">
-        <v>170100</v>
-      </c>
-      <c r="E2" t="n">
-        <v>46100</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2011</v>
-      </c>
-      <c r="B3" t="n">
-        <v>164300</v>
       </c>
       <c r="C3" t="n">
         <v>505400</v>
       </c>
       <c r="D3" t="n">
+        <v>496100</v>
+      </c>
+      <c r="E3" t="n">
+        <v>497000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>505800</v>
+      </c>
+      <c r="G3" t="n">
+        <v>535100</v>
+      </c>
+      <c r="H3" t="n">
+        <v>552000</v>
+      </c>
+      <c r="I3" t="n">
+        <v>572800</v>
+      </c>
+      <c r="J3" t="n">
+        <v>593200</v>
+      </c>
+      <c r="K3" t="n">
+        <v>640400</v>
+      </c>
+      <c r="L3" t="n">
+        <v>680800</v>
+      </c>
+      <c r="M3" t="n">
+        <v>712400</v>
+      </c>
+      <c r="N3" t="n">
+        <v>746400</v>
+      </c>
+      <c r="O3" t="n">
+        <v>771700</v>
+      </c>
+      <c r="P3" t="n">
+        <v>797900</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>819900</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vocational education</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>46100</v>
+      </c>
+      <c r="C4" t="n">
+        <v>48100</v>
+      </c>
+      <c r="D4" t="n">
+        <v>45300</v>
+      </c>
+      <c r="E4" t="n">
+        <v>42800</v>
+      </c>
+      <c r="F4" t="n">
+        <v>42800</v>
+      </c>
+      <c r="G4" t="n">
+        <v>42700</v>
+      </c>
+      <c r="H4" t="n">
+        <v>40100</v>
+      </c>
+      <c r="I4" t="n">
+        <v>35800</v>
+      </c>
+      <c r="J4" t="n">
+        <v>37000</v>
+      </c>
+      <c r="K4" t="n">
+        <v>37800</v>
+      </c>
+      <c r="L4" t="n">
+        <v>40200</v>
+      </c>
+      <c r="M4" t="n">
+        <v>42600</v>
+      </c>
+      <c r="N4" t="n">
+        <v>38000</v>
+      </c>
+      <c r="O4" t="n">
+        <v>38300</v>
+      </c>
+      <c r="P4" t="n">
+        <v>40900</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>41600</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Higher education</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>170100</v>
+      </c>
+      <c r="C5" t="n">
         <v>172800</v>
       </c>
-      <c r="E3" t="n">
-        <v>48100</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2012</v>
-      </c>
-      <c r="B4" t="n">
-        <v>181000</v>
-      </c>
-      <c r="C4" t="n">
-        <v>496100</v>
-      </c>
-      <c r="D4" t="n">
+      <c r="D5" t="n">
         <v>175500</v>
       </c>
-      <c r="E4" t="n">
-        <v>45300</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2013</v>
-      </c>
-      <c r="B5" t="n">
-        <v>193700</v>
-      </c>
-      <c r="C5" t="n">
-        <v>497000</v>
-      </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>174100</v>
       </c>
-      <c r="E5" t="n">
-        <v>42800</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2014</v>
-      </c>
-      <c r="B6" t="n">
-        <v>206600</v>
-      </c>
-      <c r="C6" t="n">
-        <v>505800</v>
-      </c>
-      <c r="D6" t="n">
+      <c r="F5" t="n">
         <v>178300</v>
       </c>
-      <c r="E6" t="n">
-        <v>42800</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B7" t="n">
-        <v>225400</v>
-      </c>
-      <c r="C7" t="n">
-        <v>535100</v>
-      </c>
-      <c r="D7" t="n">
+      <c r="G5" t="n">
         <v>162600</v>
       </c>
-      <c r="E7" t="n">
-        <v>42700</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B8" t="n">
-        <v>243400</v>
-      </c>
-      <c r="C8" t="n">
-        <v>552000</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="H5" t="n">
         <v>157100</v>
       </c>
-      <c r="E8" t="n">
-        <v>40100</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B9" t="n">
-        <v>256700</v>
-      </c>
-      <c r="C9" t="n">
-        <v>572800</v>
-      </c>
-      <c r="D9" t="n">
+      <c r="I5" t="n">
         <v>155200</v>
       </c>
-      <c r="E9" t="n">
-        <v>35800</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B10" t="n">
-        <v>261300</v>
-      </c>
-      <c r="C10" t="n">
-        <v>593200</v>
-      </c>
-      <c r="D10" t="n">
+      <c r="J5" t="n">
         <v>157600</v>
       </c>
-      <c r="E10" t="n">
-        <v>37000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B11" t="n">
-        <v>263300</v>
-      </c>
-      <c r="C11" t="n">
-        <v>640400</v>
-      </c>
-      <c r="D11" t="n">
+      <c r="K5" t="n">
         <v>148400</v>
       </c>
-      <c r="E11" t="n">
-        <v>37800</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B12" t="n">
-        <v>247000</v>
-      </c>
-      <c r="C12" t="n">
-        <v>680800</v>
-      </c>
-      <c r="D12" t="n">
+      <c r="L5" t="n">
         <v>147300</v>
       </c>
-      <c r="E12" t="n">
-        <v>40200</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B13" t="n">
-        <v>191000</v>
-      </c>
-      <c r="C13" t="n">
-        <v>712400</v>
-      </c>
-      <c r="D13" t="n">
+      <c r="M5" t="n">
         <v>149000</v>
       </c>
-      <c r="E13" t="n">
-        <v>42600</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B14" t="n">
-        <v>266000</v>
-      </c>
-      <c r="C14" t="n">
-        <v>746400</v>
-      </c>
-      <c r="D14" t="n">
+      <c r="N5" t="n">
         <v>145300</v>
       </c>
-      <c r="E14" t="n">
-        <v>38000</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B15" t="n">
-        <v>274200</v>
-      </c>
-      <c r="C15" t="n">
-        <v>771700</v>
-      </c>
-      <c r="D15" t="n">
+      <c r="O5" t="n">
         <v>145300</v>
       </c>
-      <c r="E15" t="n">
-        <v>38300</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B16" t="n">
-        <v>264800</v>
-      </c>
-      <c r="C16" t="n">
-        <v>797900</v>
-      </c>
-      <c r="D16" t="n">
+      <c r="P5" t="n">
         <v>150300</v>
       </c>
-      <c r="E16" t="n">
-        <v>40900</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B17" t="n">
-        <v>258800</v>
-      </c>
-      <c r="C17" t="n">
-        <v>819900</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="Q5" t="n">
         <v>161900</v>
-      </c>
-      <c r="E17" t="n">
-        <v>41600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>